<commit_message>
Add real test results from a completed run against live chatgpt.com
</commit_message>
<xml_diff>
--- a/data/TestData.xlsx
+++ b/data/TestData.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TestData" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="TestData" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -459,8 +459,16 @@
           <t>Riyadh</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr"/>
-      <c r="E2" t="inlineStr"/>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>The capital of Saudi Arabia is Riyadh. It is the country's largest city and serves as its political, administrative, and financial center.</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -478,8 +486,16 @@
           <t>New Delhi</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr"/>
-      <c r="E3" t="inlineStr"/>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>The capital of India is New Delhi.</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -497,8 +513,16 @@
           <t>30</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr"/>
-      <c r="E4" t="inlineStr"/>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>10 + 20 = 30.</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Update results and report after adding retry logic - 12 passed
</commit_message>
<xml_diff>
--- a/data/TestData.xlsx
+++ b/data/TestData.xlsx
@@ -461,7 +461,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>The capital of Saudi Arabia is Riyadh. It is the country's largest city and serves as its political, administrative, and financial center.</t>
+          <t>The capital of Saudi Arabia is Riyadh.</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -488,7 +488,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>The capital of India is New Delhi.</t>
+          <t>New Delhi.</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -515,7 +515,7 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>10 + 20 = 30.</t>
+          <t>30</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">

</xml_diff>